<commit_message>
fixed demand to IRP2025 LOWDelEVs
</commit_message>
<xml_diff>
--- a/scenarios/Coal_Flexibilisation/sub_scenarios/annual_load.xlsx
+++ b/scenarios/Coal_Flexibilisation/sub_scenarios/annual_load.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\agatha.majcher\Downloads\agma0 pypsa-rsa master scenarios-Coal_Flexibilisation\sub_scenarios\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rlinstitutde-my.sharepoint.com/personal/agatha_majcher_rl-institut_de/Documents/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFEF3B16-1B2E-4765-A4C2-FF1C1AE5C7DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="80" documentId="13_ncr:1_{DFEF3B16-1B2E-4765-A4C2-FF1C1AE5C7DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4C02FBF7-7246-4068-B1EE-7CD838C0D288}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -50,20 +50,21 @@
     <t>TWh/a</t>
   </si>
   <si>
-    <t>CAGR 2040-2050 extended</t>
+    <t>IRP2025(UCT)</t>
   </si>
   <si>
-    <t>IRP24_MOD</t>
+    <t>LOWDelEVs</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="#,##0.000"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -108,14 +109,8 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF555D6A"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -141,8 +136,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.79998168889431442"/>
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor theme="9" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor theme="9" tint="0.79998168889431442"/>
       </patternFill>
     </fill>
   </fills>
@@ -194,9 +201,15 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -210,22 +223,23 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="1" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -516,188 +530,190 @@
   <cols>
     <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="28" width="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="28" width="7.5703125" bestFit="1" customWidth="1"/>
     <col min="29" max="29" width="24.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3">
+      <c r="C1" s="7">
         <v>2025</v>
       </c>
-      <c r="D1" s="3">
+      <c r="D1" s="7">
         <v>2026</v>
       </c>
-      <c r="E1" s="3">
+      <c r="E1" s="7">
         <v>2027</v>
       </c>
-      <c r="F1" s="3">
+      <c r="F1" s="7">
         <v>2028</v>
       </c>
-      <c r="G1" s="3">
+      <c r="G1" s="7">
         <v>2029</v>
       </c>
-      <c r="H1" s="3">
+      <c r="H1" s="7">
         <v>2030</v>
       </c>
-      <c r="I1" s="3">
+      <c r="I1" s="7">
         <v>2031</v>
       </c>
-      <c r="J1" s="3">
+      <c r="J1" s="7">
         <v>2032</v>
       </c>
-      <c r="K1" s="3">
+      <c r="K1" s="7">
         <v>2033</v>
       </c>
-      <c r="L1" s="3">
+      <c r="L1" s="7">
         <v>2034</v>
       </c>
-      <c r="M1" s="3">
+      <c r="M1" s="7">
         <v>2035</v>
       </c>
-      <c r="N1" s="3">
+      <c r="N1" s="7">
         <v>2036</v>
       </c>
-      <c r="O1" s="3">
+      <c r="O1" s="7">
         <v>2037</v>
       </c>
-      <c r="P1" s="3">
+      <c r="P1" s="7">
         <v>2038</v>
       </c>
-      <c r="Q1" s="3">
+      <c r="Q1" s="7">
         <v>2039</v>
       </c>
-      <c r="R1" s="3">
+      <c r="R1" s="7">
         <v>2040</v>
       </c>
-      <c r="S1" s="3">
+      <c r="S1" s="7">
         <v>2041</v>
       </c>
-      <c r="T1" s="3">
+      <c r="T1" s="7">
         <v>2042</v>
       </c>
-      <c r="U1" s="3">
+      <c r="U1" s="7">
         <v>2043</v>
       </c>
-      <c r="V1" s="3">
+      <c r="V1" s="7">
         <v>2044</v>
       </c>
-      <c r="W1" s="3">
+      <c r="W1" s="7">
         <v>2045</v>
       </c>
-      <c r="X1" s="3">
+      <c r="X1" s="7">
         <v>2046</v>
       </c>
-      <c r="Y1" s="3">
+      <c r="Y1" s="7">
         <v>2047</v>
       </c>
-      <c r="Z1" s="3">
+      <c r="Z1" s="7">
         <v>2048</v>
       </c>
-      <c r="AA1" s="3">
+      <c r="AA1" s="7">
         <v>2049</v>
       </c>
-      <c r="AB1" s="3">
+      <c r="AB1" s="7">
         <v>2050</v>
       </c>
-      <c r="AC1" s="3" t="s">
+      <c r="AC1" s="7" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="1">
-        <v>240.13551922508401</v>
-      </c>
-      <c r="D2" s="1">
-        <v>242.136474226335</v>
-      </c>
-      <c r="E2" s="1">
-        <v>246.26344391641399</v>
-      </c>
-      <c r="F2" s="1">
-        <v>250.265353918915</v>
-      </c>
-      <c r="G2" s="1">
-        <v>254.64244298415099</v>
-      </c>
-      <c r="H2" s="1">
-        <v>260.770367675481</v>
-      </c>
-      <c r="I2" s="1">
-        <v>268.89924736806199</v>
-      </c>
-      <c r="J2" s="1">
-        <v>277.40330612337698</v>
-      </c>
-      <c r="K2" s="1">
-        <v>283.28111143954999</v>
-      </c>
-      <c r="L2" s="1">
-        <v>290.53457331908402</v>
-      </c>
-      <c r="M2" s="1">
-        <v>298.66345301166399</v>
-      </c>
-      <c r="N2" s="1">
-        <v>305.541735828463</v>
-      </c>
-      <c r="O2" s="1">
-        <v>313.04531708315301</v>
-      </c>
-      <c r="P2" s="1">
-        <v>321.67443552604601</v>
-      </c>
-      <c r="Q2" s="1">
-        <v>330.80379271925199</v>
-      </c>
-      <c r="R2" s="1">
-        <v>339.93314991245802</v>
-      </c>
-      <c r="S2" s="1">
-        <v>347.93696991745998</v>
-      </c>
-      <c r="T2" s="1">
-        <v>357.56656586097898</v>
-      </c>
-      <c r="U2" s="1">
-        <v>366.19568430387199</v>
-      </c>
-      <c r="V2" s="1">
-        <v>376.325518997703</v>
-      </c>
-      <c r="W2" s="1">
-        <v>384.32933900270501</v>
-      </c>
-      <c r="X2" s="1">
-        <v>391.95797994497298</v>
-      </c>
-      <c r="Y2" s="1">
-        <v>403.21335182700801</v>
-      </c>
-      <c r="Z2" s="1">
-        <v>413.09306714568299</v>
-      </c>
-      <c r="AA2" s="1">
-        <v>419.97134996248201</v>
-      </c>
-      <c r="AB2" s="1">
-        <v>430.60142340662497</v>
-      </c>
-      <c r="AC2" s="1" t="s">
+      <c r="C2" s="3">
+        <v>228.53899999999999</v>
+      </c>
+      <c r="D2" s="3">
+        <v>231.089</v>
+      </c>
+      <c r="E2" s="3">
+        <v>231.47</v>
+      </c>
+      <c r="F2" s="4">
+        <v>231.65600000000001</v>
+      </c>
+      <c r="G2" s="5">
+        <v>232.37200000000001</v>
+      </c>
+      <c r="H2" s="4">
+        <v>235.36600000000001</v>
+      </c>
+      <c r="I2" s="5">
+        <v>238.90100000000001</v>
+      </c>
+      <c r="J2" s="4">
+        <v>242.65799999999999</v>
+      </c>
+      <c r="K2" s="5">
+        <v>247.172</v>
+      </c>
+      <c r="L2" s="4">
+        <v>252.77600000000001</v>
+      </c>
+      <c r="M2" s="5">
+        <v>258.80700000000002</v>
+      </c>
+      <c r="N2" s="4">
+        <v>264.68200000000002</v>
+      </c>
+      <c r="O2" s="5">
+        <v>271.14999999999998</v>
+      </c>
+      <c r="P2" s="4">
+        <v>277.64699999999999</v>
+      </c>
+      <c r="Q2" s="5">
+        <v>284.18700000000001</v>
+      </c>
+      <c r="R2" s="4">
+        <v>291.12799999999999</v>
+      </c>
+      <c r="S2" s="5">
+        <v>298.77199999999999</v>
+      </c>
+      <c r="T2" s="4">
+        <v>306.66899999999998</v>
+      </c>
+      <c r="U2" s="5">
+        <v>316.21100000000001</v>
+      </c>
+      <c r="V2" s="4">
+        <v>323.81200000000001</v>
+      </c>
+      <c r="W2" s="5">
+        <v>331.84100000000001</v>
+      </c>
+      <c r="X2" s="4">
+        <v>341.32600000000002</v>
+      </c>
+      <c r="Y2" s="5">
+        <v>351.46600000000001</v>
+      </c>
+      <c r="Z2" s="4">
+        <v>358.553</v>
+      </c>
+      <c r="AA2" s="5">
+        <v>368.16899999999998</v>
+      </c>
+      <c r="AB2" s="4">
+        <v>378.56099999999998</v>
+      </c>
+      <c r="AC2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="AD2" s="4"/>
+      <c r="AD2" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>